<commit_message>
Ship name edits, minor methods edits
</commit_message>
<xml_diff>
--- a/nutrient-mvco-info.xlsx
+++ b/nutrient-mvco-info.xlsx
@@ -1,16 +1,16 @@
 
 <file path=xl/workbook.xml><?xml version="1.0" encoding="utf-8"?>
 <workbook xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x15="http://schemas.microsoft.com/office/spreadsheetml/2010/11/main" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr6="http://schemas.microsoft.com/office/spreadsheetml/2016/revision6" xmlns:xr10="http://schemas.microsoft.com/office/spreadsheetml/2016/revision10" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" mc:Ignorable="x15 xr xr6 xr10 xr2">
-  <fileVersion appName="xl" lastEdited="7" lowestEdited="6" rupBuild="27726"/>
+  <fileVersion appName="xl" lastEdited="7" lowestEdited="6" rupBuild="30228"/>
   <workbookPr/>
   <mc:AlternateContent xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006">
     <mc:Choice Requires="x15">
-      <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="C:\Users\wanglab\Documents\GitHub\nes-lter-nutrient\"/>
+      <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="C:\Users\kmorkeski\Documents\nes-lter-nutrient-mvco\"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{15B29A38-CF49-4913-A1AE-6C610EBA87C0}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
+  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{238D9A0E-90E0-4467-BA75-29B0D7FF3AA9}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
   <bookViews>
-    <workbookView xWindow="28680" yWindow="-120" windowWidth="29040" windowHeight="17640" xr2:uid="{00000000-000D-0000-FFFF-FFFF00000000}"/>
+    <workbookView xWindow="36180" yWindow="6825" windowWidth="21600" windowHeight="10695" activeTab="3" xr2:uid="{00000000-000D-0000-FFFF-FFFF00000000}"/>
   </bookViews>
   <sheets>
     <sheet name="ColumnHeaders" sheetId="1" r:id="rId1"/>
@@ -28,7 +28,7 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="171" uniqueCount="97">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="172" uniqueCount="102">
   <si>
     <t>attributeName</t>
   </si>
@@ -198,15 +198,9 @@
     <t>NSF</t>
   </si>
   <si>
-    <t>OCE-1655686</t>
-  </si>
-  <si>
     <t>creator</t>
   </si>
   <si>
-    <t>E. Taylor</t>
-  </si>
-  <si>
     <t>Crockford</t>
   </si>
   <si>
@@ -319,13 +313,34 @@
   </si>
   <si>
     <t>date_time_utc</t>
+  </si>
+  <si>
+    <t xml:space="preserve">E. </t>
+  </si>
+  <si>
+    <t>Taylor</t>
+  </si>
+  <si>
+    <t>OCE-2322676</t>
+  </si>
+  <si>
+    <t>OCE-2322677</t>
+  </si>
+  <si>
+    <t>OCE-2322678</t>
+  </si>
+  <si>
+    <t>OCE-2322679</t>
+  </si>
+  <si>
+    <t>OCE-2322680</t>
   </si>
 </sst>
 </file>
 
 <file path=xl/styles.xml><?xml version="1.0" encoding="utf-8"?>
 <styleSheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:x16r2="http://schemas.microsoft.com/office/spreadsheetml/2015/02/main" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" mc:Ignorable="x14ac x16r2 xr">
-  <fonts count="4" x14ac:knownFonts="1">
+  <fonts count="5" x14ac:knownFonts="1">
     <font>
       <sz val="11"/>
       <color theme="1"/>
@@ -350,6 +365,12 @@
     <font>
       <sz val="11"/>
       <color rgb="FF000000"/>
+      <name val="Calibri"/>
+      <family val="2"/>
+      <scheme val="minor"/>
+    </font>
+    <font>
+      <sz val="8"/>
       <name val="Calibri"/>
       <family val="2"/>
       <scheme val="minor"/>
@@ -704,61 +725,61 @@
     </row>
     <row r="2" spans="1:7" x14ac:dyDescent="0.3">
       <c r="A2" t="s">
-        <v>64</v>
+        <v>62</v>
       </c>
       <c r="B2" s="5" t="s">
-        <v>93</v>
+        <v>91</v>
       </c>
       <c r="C2" t="s">
         <v>9</v>
       </c>
       <c r="F2" t="s">
-        <v>87</v>
+        <v>85</v>
       </c>
       <c r="G2" t="s">
-        <v>87</v>
+        <v>85</v>
       </c>
     </row>
     <row r="3" spans="1:7" x14ac:dyDescent="0.3">
       <c r="A3" t="s">
-        <v>65</v>
+        <v>63</v>
       </c>
       <c r="B3" s="5" t="s">
-        <v>94</v>
+        <v>92</v>
       </c>
       <c r="C3" t="s">
         <v>9</v>
       </c>
       <c r="F3" t="s">
-        <v>87</v>
+        <v>85</v>
       </c>
       <c r="G3" t="s">
-        <v>87</v>
+        <v>85</v>
       </c>
     </row>
     <row r="4" spans="1:7" x14ac:dyDescent="0.3">
       <c r="A4" t="s">
-        <v>76</v>
+        <v>74</v>
       </c>
       <c r="B4" s="1" t="s">
-        <v>77</v>
+        <v>75</v>
       </c>
       <c r="C4" t="s">
         <v>9</v>
       </c>
       <c r="F4" t="s">
-        <v>87</v>
+        <v>85</v>
       </c>
       <c r="G4" t="s">
-        <v>87</v>
+        <v>85</v>
       </c>
     </row>
     <row r="5" spans="1:7" x14ac:dyDescent="0.3">
       <c r="A5" t="s">
-        <v>95</v>
+        <v>93</v>
       </c>
       <c r="B5" s="1" t="s">
-        <v>92</v>
+        <v>90</v>
       </c>
       <c r="C5" t="s">
         <v>9</v>
@@ -766,22 +787,22 @@
     </row>
     <row r="6" spans="1:7" x14ac:dyDescent="0.3">
       <c r="A6" t="s">
-        <v>96</v>
+        <v>94</v>
       </c>
       <c r="B6" s="1" t="s">
-        <v>73</v>
+        <v>71</v>
       </c>
       <c r="C6" t="s">
         <v>7</v>
       </c>
       <c r="E6" t="s">
-        <v>63</v>
+        <v>61</v>
       </c>
       <c r="F6" t="s">
-        <v>87</v>
+        <v>85</v>
       </c>
       <c r="G6" t="s">
-        <v>87</v>
+        <v>85</v>
       </c>
     </row>
     <row r="7" spans="1:7" x14ac:dyDescent="0.3">
@@ -789,7 +810,7 @@
         <v>11</v>
       </c>
       <c r="B7" s="1" t="s">
-        <v>85</v>
+        <v>83</v>
       </c>
       <c r="C7" t="s">
         <v>10</v>
@@ -798,7 +819,7 @@
         <v>22</v>
       </c>
       <c r="F7" t="s">
-        <v>88</v>
+        <v>86</v>
       </c>
       <c r="G7" t="s">
         <v>8</v>
@@ -809,7 +830,7 @@
         <v>12</v>
       </c>
       <c r="B8" s="1" t="s">
-        <v>86</v>
+        <v>84</v>
       </c>
       <c r="C8" t="s">
         <v>10</v>
@@ -818,7 +839,7 @@
         <v>22</v>
       </c>
       <c r="F8" t="s">
-        <v>88</v>
+        <v>86</v>
       </c>
       <c r="G8" t="s">
         <v>8</v>
@@ -838,7 +859,7 @@
         <v>23</v>
       </c>
       <c r="F9" t="s">
-        <v>88</v>
+        <v>86</v>
       </c>
       <c r="G9" t="s">
         <v>8</v>
@@ -849,16 +870,16 @@
         <v>14</v>
       </c>
       <c r="B10" s="1" t="s">
-        <v>66</v>
+        <v>64</v>
       </c>
       <c r="C10" t="s">
         <v>9</v>
       </c>
       <c r="F10" t="s">
-        <v>87</v>
+        <v>85</v>
       </c>
       <c r="G10" t="s">
-        <v>87</v>
+        <v>85</v>
       </c>
     </row>
     <row r="11" spans="1:7" ht="28.8" x14ac:dyDescent="0.3">
@@ -875,7 +896,7 @@
         <v>24</v>
       </c>
       <c r="F11" t="s">
-        <v>88</v>
+        <v>86</v>
       </c>
       <c r="G11" t="s">
         <v>8</v>
@@ -886,7 +907,7 @@
         <v>16</v>
       </c>
       <c r="B12" s="1" t="s">
-        <v>74</v>
+        <v>72</v>
       </c>
       <c r="C12" t="s">
         <v>10</v>
@@ -895,7 +916,7 @@
         <v>24</v>
       </c>
       <c r="F12" t="s">
-        <v>88</v>
+        <v>86</v>
       </c>
       <c r="G12" t="s">
         <v>8</v>
@@ -906,7 +927,7 @@
         <v>18</v>
       </c>
       <c r="B13" s="1" t="s">
-        <v>75</v>
+        <v>73</v>
       </c>
       <c r="C13" t="s">
         <v>10</v>
@@ -915,7 +936,7 @@
         <v>24</v>
       </c>
       <c r="F13" t="s">
-        <v>88</v>
+        <v>86</v>
       </c>
       <c r="G13" t="s">
         <v>8</v>
@@ -935,7 +956,7 @@
         <v>24</v>
       </c>
       <c r="F14" t="s">
-        <v>88</v>
+        <v>86</v>
       </c>
       <c r="G14" t="s">
         <v>8</v>
@@ -943,13 +964,13 @@
     </row>
     <row r="15" spans="1:7" x14ac:dyDescent="0.3">
       <c r="A15" t="s">
-        <v>80</v>
+        <v>78</v>
       </c>
       <c r="B15" t="s">
-        <v>78</v>
+        <v>76</v>
       </c>
       <c r="C15" s="6" t="s">
-        <v>79</v>
+        <v>77</v>
       </c>
     </row>
     <row r="21" spans="2:2" ht="15.6" x14ac:dyDescent="0.3">
@@ -1021,7 +1042,7 @@
         <v>54</v>
       </c>
       <c r="G2" t="s">
-        <v>57</v>
+        <v>56</v>
       </c>
       <c r="H2" t="s">
         <v>52</v>
@@ -1030,7 +1051,7 @@
         <v>55</v>
       </c>
       <c r="J2" t="s">
-        <v>56</v>
+        <v>97</v>
       </c>
     </row>
     <row r="3" spans="1:10" x14ac:dyDescent="0.3">
@@ -1053,7 +1074,7 @@
         <v>54</v>
       </c>
       <c r="G3" t="s">
-        <v>67</v>
+        <v>65</v>
       </c>
       <c r="H3" t="s">
         <v>52</v>
@@ -1062,27 +1083,30 @@
         <v>55</v>
       </c>
       <c r="J3" t="s">
-        <v>56</v>
+        <v>98</v>
       </c>
     </row>
     <row r="4" spans="1:10" x14ac:dyDescent="0.3">
       <c r="A4" t="s">
-        <v>58</v>
+        <v>95</v>
+      </c>
+      <c r="B4" t="s">
+        <v>96</v>
       </c>
       <c r="C4" t="s">
-        <v>59</v>
+        <v>57</v>
       </c>
       <c r="D4" t="s">
         <v>52</v>
       </c>
       <c r="E4" t="s">
-        <v>71</v>
+        <v>69</v>
       </c>
       <c r="F4" t="s">
-        <v>89</v>
+        <v>87</v>
       </c>
       <c r="G4" t="s">
-        <v>57</v>
+        <v>56</v>
       </c>
       <c r="H4" t="s">
         <v>52</v>
@@ -1091,27 +1115,27 @@
         <v>55</v>
       </c>
       <c r="J4" t="s">
-        <v>56</v>
+        <v>99</v>
       </c>
     </row>
     <row r="5" spans="1:10" x14ac:dyDescent="0.3">
       <c r="A5" t="s">
-        <v>68</v>
+        <v>66</v>
       </c>
       <c r="C5" t="s">
-        <v>69</v>
+        <v>67</v>
       </c>
       <c r="D5" t="s">
         <v>52</v>
       </c>
       <c r="E5" t="s">
-        <v>70</v>
+        <v>68</v>
       </c>
       <c r="F5" t="s">
-        <v>90</v>
+        <v>88</v>
       </c>
       <c r="G5" t="s">
-        <v>57</v>
+        <v>56</v>
       </c>
       <c r="H5" t="s">
         <v>52</v>
@@ -1120,21 +1144,21 @@
         <v>55</v>
       </c>
       <c r="J5" t="s">
-        <v>56</v>
+        <v>100</v>
       </c>
     </row>
     <row r="6" spans="1:10" x14ac:dyDescent="0.3">
       <c r="A6" t="s">
-        <v>60</v>
+        <v>58</v>
       </c>
       <c r="D6" t="s">
         <v>52</v>
       </c>
       <c r="E6" t="s">
-        <v>61</v>
+        <v>59</v>
       </c>
       <c r="G6" t="s">
-        <v>62</v>
+        <v>60</v>
       </c>
       <c r="H6" t="s">
         <v>52</v>
@@ -1143,10 +1167,11 @@
         <v>55</v>
       </c>
       <c r="J6" t="s">
-        <v>56</v>
+        <v>101</v>
       </c>
     </row>
   </sheetData>
+  <phoneticPr fontId="4" type="noConversion"/>
   <pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
 </worksheet>
 </file>
@@ -1170,7 +1195,7 @@
     </row>
     <row r="2" spans="1:2" x14ac:dyDescent="0.3">
       <c r="A2" t="s">
-        <v>72</v>
+        <v>70</v>
       </c>
       <c r="B2" t="s">
         <v>27</v>
@@ -1285,43 +1310,43 @@
         <v>0</v>
       </c>
       <c r="B1" s="4" t="s">
-        <v>81</v>
+        <v>79</v>
       </c>
       <c r="C1" s="4" t="s">
-        <v>82</v>
+        <v>80</v>
       </c>
     </row>
     <row r="2" spans="1:3" x14ac:dyDescent="0.3">
       <c r="A2" t="s">
-        <v>80</v>
+        <v>78</v>
       </c>
       <c r="B2" s="4">
         <v>1</v>
       </c>
       <c r="C2" s="4" t="s">
-        <v>83</v>
+        <v>81</v>
       </c>
     </row>
     <row r="3" spans="1:3" x14ac:dyDescent="0.3">
       <c r="A3" t="s">
-        <v>80</v>
+        <v>78</v>
       </c>
       <c r="B3" s="4">
         <v>2</v>
       </c>
       <c r="C3" t="s">
-        <v>91</v>
+        <v>89</v>
       </c>
     </row>
     <row r="4" spans="1:3" x14ac:dyDescent="0.3">
       <c r="A4" t="s">
-        <v>80</v>
+        <v>78</v>
       </c>
       <c r="B4" s="4">
         <v>3</v>
       </c>
       <c r="C4" s="4" t="s">
-        <v>84</v>
+        <v>82</v>
       </c>
     </row>
   </sheetData>

</xml_diff>